<commit_message>
feat: enhance module extraction and selection process; improve stability metrics and logging
</commit_message>
<xml_diff>
--- a/info table.xlsx
+++ b/info table.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23028" windowHeight="9780"/>
+    <workbookView windowWidth="20544" windowHeight="9588"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="88">
   <si>
     <t>Основные источники данных:</t>
   </si>
@@ -186,18 +186,127 @@
   </si>
   <si>
     <t>SETD2</t>
+  </si>
+  <si>
+    <t>Starting time</t>
+  </si>
+  <si>
+    <t>k=6 with 20 subsampling iterations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stability score: 0.828  </t>
+  </si>
+  <si>
+    <t>k=8 with 20 subsampling iterations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stability score: 0.869 </t>
+  </si>
+  <si>
+    <t>ДАННЫЕ ТОЛЬКО С TCGA НУЖНА ДОП ВАЛИДАЦИЯ</t>
+  </si>
+  <si>
+    <t>Modules</t>
+  </si>
+  <si>
+    <t>Смотрим по кол-ву процентной частоте встречи мутации у онкобольных</t>
+  </si>
+  <si>
+    <t>Module 0</t>
+  </si>
+  <si>
+    <t>APC, FBXW7, TCF7L2, SOX9, SMAD4, TP53, AMER1, NRAS</t>
+  </si>
+  <si>
+    <t>Brain modules</t>
+  </si>
+  <si>
+    <t>TP53, IDH1, ATRX, PTEN, MUC16, EGFR, PIK3CA, NF1, BRAF, CIC</t>
+  </si>
+  <si>
+    <t>Module 1</t>
+  </si>
+  <si>
+    <t>CDKN2A, CDKN2Ap16INK4A, SMAD4, TP53, PTPRT, FAT1, ERBB4, NOTCH1</t>
+  </si>
+  <si>
+    <t>Eye modules</t>
+  </si>
+  <si>
+    <t>GNAQ, GNA11, SF3B1, FGFR4, BAP1, EIF1AX, BCOR, MUC16, NF1, LRP1B</t>
+  </si>
+  <si>
+    <t>Module 2</t>
+  </si>
+  <si>
+    <t>NF1, FAT1, PTPRD, PTPRT, GRIN2A, ROS1, ERBB4, ATM</t>
+  </si>
+  <si>
+    <t>Thyroid (гланды)</t>
+  </si>
+  <si>
+    <t>BRAF, NRAS, HRAS, MUC16, ZFHX3, EIF1AX, DICER, KMT2A, AKT1, ATM</t>
+  </si>
+  <si>
+    <t>Module 3</t>
+  </si>
+  <si>
+    <t>ARID1A, PTEN, KMT2D, ZFHX3, KMT2B, PIK3R1, CTCF, CTNNB1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lymph Nodes </t>
+  </si>
+  <si>
+    <t>MUC16, BRAF, LRP1B, CSMD3, FAT4, FAT3, PTPRT, GRIN2A, FAM135B, CNTNAP2</t>
+  </si>
+  <si>
+    <t>Module 4</t>
+  </si>
+  <si>
+    <t>TP53, RB1, EGFR, ATRX, NF1, MLL2, PTPRD, EPHA5</t>
+  </si>
+  <si>
+    <t>Esophagus</t>
+  </si>
+  <si>
+    <t>TP53, MUC16, LRP1B, CSMD3, FAT3, FAT4, KMT2D, CDKN2A, ARID1A, NOTCH1</t>
+  </si>
+  <si>
+    <t>Module 5</t>
+  </si>
+  <si>
+    <t>PIK3CA, CDH1, MAP3K1, GATA3, FBXW7, FOXA1, CTNNB1, KDM6A</t>
+  </si>
+  <si>
+    <t>Soft tissue</t>
+  </si>
+  <si>
+    <t>MUC16, TP53, LRP1B, CSMD3, FAT4, FAT3, GRIN2A, NRAS, PTPRT, DCC1</t>
+  </si>
+  <si>
+    <t>Module 6</t>
+  </si>
+  <si>
+    <t>KRAS, SMAD4, STK11, ATM, RBM10, KEAP1, GNAS, TGFBR2</t>
+  </si>
+  <si>
+    <t>Module 7</t>
+  </si>
+  <si>
+    <t>TERT, BRAF, NRAS, KDM6A, FGFR3, KMT2D, RB1, PTPRT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="_-* #,##0.00\ &quot;₽&quot;_-;\-* #,##0.00\ &quot;₽&quot;_-;_-* &quot;-&quot;??\ &quot;₽&quot;_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-* #,##0\ &quot;₽&quot;_-;\-* #,##0\ &quot;₽&quot;_-;_-* &quot;-&quot;\ &quot;₽&quot;_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="179" formatCode="dd\.mm\.yyyy\ h:mm"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -815,7 +924,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -838,6 +947,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1365,7 +1477,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B3:H40"/>
+  <dimension ref="B3:H60"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="28.6666666666667" customWidth="1"/>
@@ -1419,7 +1531,6 @@
       <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="C7"/>
       <c r="D7" t="s">
         <v>10</v>
       </c>
@@ -1612,6 +1723,143 @@
     <row r="40" spans="2:5">
       <c r="C40" t="s">
         <v>51</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5">
+      <c r="B48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7">
+      <c r="B49" s="8">
+        <v>46288.5851967593</v>
+      </c>
+      <c r="D49" t="s">
+        <v>53</v>
+      </c>
+      <c r="E49" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7">
+      <c r="D50" t="s">
+        <v>55</v>
+      </c>
+      <c r="E50" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7">
+      <c r="F51" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7">
+      <c r="B52" t="s">
+        <v>58</v>
+      </c>
+      <c r="F52" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7">
+      <c r="B53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C53" t="s">
+        <v>61</v>
+      </c>
+      <c r="F53" t="s">
+        <v>62</v>
+      </c>
+      <c r="G53" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7">
+      <c r="B54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C54" t="s">
+        <v>65</v>
+      </c>
+      <c r="F54" t="s">
+        <v>66</v>
+      </c>
+      <c r="G54" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7">
+      <c r="B55" t="s">
+        <v>68</v>
+      </c>
+      <c r="C55" t="s">
+        <v>69</v>
+      </c>
+      <c r="F55" t="s">
+        <v>70</v>
+      </c>
+      <c r="G55" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7">
+      <c r="B56" t="s">
+        <v>72</v>
+      </c>
+      <c r="C56" t="s">
+        <v>73</v>
+      </c>
+      <c r="F56" t="s">
+        <v>74</v>
+      </c>
+      <c r="G56" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7">
+      <c r="B57" t="s">
+        <v>76</v>
+      </c>
+      <c r="C57" t="s">
+        <v>77</v>
+      </c>
+      <c r="F57" t="s">
+        <v>78</v>
+      </c>
+      <c r="G57" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7">
+      <c r="B58" t="s">
+        <v>80</v>
+      </c>
+      <c r="C58" t="s">
+        <v>81</v>
+      </c>
+      <c r="F58" t="s">
+        <v>82</v>
+      </c>
+      <c r="G58" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7">
+      <c r="B59" t="s">
+        <v>84</v>
+      </c>
+      <c r="C59" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7">
+      <c r="B60" t="s">
+        <v>86</v>
+      </c>
+      <c r="C60" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>